<commit_message>
fix: close template integrity gaps
</commit_message>
<xml_diff>
--- a/library/templates/TMPL-0001/1.0.0/internal-close-reconciliation.xlsx
+++ b/library/templates/TMPL-0001/1.0.0/internal-close-reconciliation.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Close_Control" sheetId="1" r:id="R7d797c8c49a948ea"/>
-    <sheet name="Source_Data" sheetId="2" r:id="Rc0cf7d941f814d4e"/>
-    <sheet name="Account_Map" sheetId="3" r:id="Red296cad5725462d"/>
-    <sheet name="Reconciliation" sheetId="4" r:id="Rcd655485cd704ec5"/>
-    <sheet name="Proposed_Entries" sheetId="5" r:id="R0e1ca55286bd40d6"/>
-    <sheet name="Prior_Period" sheetId="6" r:id="R3f4e6bcca8ef48ba"/>
-    <sheet name="Exceptions" sheetId="7" r:id="Rbf5beb5e222e4c14"/>
-    <sheet name="Checks" sheetId="8" r:id="Raffa2827d00e44c6"/>
+    <sheet name="Close_Control" sheetId="1" r:id="R7e17d192f9f34e4c"/>
+    <sheet name="Source_Data" sheetId="2" r:id="Rdf0ddfa473394c46"/>
+    <sheet name="Account_Map" sheetId="3" r:id="R5751a82c8539442e"/>
+    <sheet name="Reconciliation" sheetId="4" r:id="R16f41c6040d141bf"/>
+    <sheet name="Proposed_Entries" sheetId="5" r:id="R18ed4b06fd0c4765"/>
+    <sheet name="Prior_Period" sheetId="6" r:id="Rb3d0f34732494bcf"/>
+    <sheet name="Exceptions" sheetId="7" r:id="Rbd3a1441b7174543"/>
+    <sheet name="Checks" sheetId="8" r:id="R85192488b71c4a2b"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Close_Control'!$A$1:$H$16</definedName>
@@ -19,7 +19,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Proposed_Entries'!$A$1:$H$19</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Prior_Period'!$A$1:$E$24</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Exceptions'!$A$1:$H$19</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="7">'Checks'!$A$1:$D$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'Checks'!$A$1:$D$14</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -376,7 +376,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="4">
+  <x:dxfs count="5">
     <x:dxf>
       <x:font>
         <x:color rgb="FF375623"/>
@@ -416,6 +416,17 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF7F6000"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -1282,7 +1293,7 @@
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
-    <tablePart r:id="R5aa5eeb5edef4e74"/>
+    <tablePart r:id="Rb83bbb3fd1194eb8"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1619,7 +1630,7 @@
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="portrait" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
-    <tablePart r:id="Rfcbc89ad489c4418"/>
+    <tablePart r:id="R81484fa93b0e4c8a"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1704,380 +1715,320 @@
     <row r="5">
       <c r="A5" s="50"/>
       <c r="B5" s="50"/>
-      <c r="C5" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A5)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A5)</f>
-        <v>0</v>
+      <c r="C5" s="67" t="str">
+        <f>IF(A5="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A5)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A5))</f>
       </c>
       <c r="D5" s="68"/>
-      <c r="E5" s="67" t="n">
-        <f>C5-D5</f>
-        <v>0</v>
+      <c r="E5" s="67" t="str">
+        <f>IF(A5="","",C5-D5)</f>
       </c>
       <c r="F5" s="68"/>
       <c r="G5" s="48" t="str">
-        <f>IF(ABS(E5)&lt;=F5,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A5="","",IF(OR(D5="",F5=""),"NOT READY",IF(ABS(E5)&lt;=F5,"PASS","REVIEW")))</f>
       </c>
       <c r="H5" s="50"/>
     </row>
     <row r="6">
       <c r="A6" s="50"/>
       <c r="B6" s="50"/>
-      <c r="C6" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A6)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A6)</f>
-        <v>0</v>
+      <c r="C6" s="67" t="str">
+        <f>IF(A6="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A6)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A6))</f>
       </c>
       <c r="D6" s="68"/>
-      <c r="E6" s="67" t="n">
-        <f>C6-D6</f>
-        <v>0</v>
+      <c r="E6" s="67" t="str">
+        <f>IF(A6="","",C6-D6)</f>
       </c>
       <c r="F6" s="68"/>
       <c r="G6" s="48" t="str">
-        <f>IF(ABS(E6)&lt;=F6,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A6="","",IF(OR(D6="",F6=""),"NOT READY",IF(ABS(E6)&lt;=F6,"PASS","REVIEW")))</f>
       </c>
       <c r="H6" s="50"/>
     </row>
     <row r="7">
       <c r="A7" s="50"/>
       <c r="B7" s="50"/>
-      <c r="C7" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A7)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A7)</f>
-        <v>0</v>
+      <c r="C7" s="67" t="str">
+        <f>IF(A7="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A7)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A7))</f>
       </c>
       <c r="D7" s="68"/>
-      <c r="E7" s="67" t="n">
-        <f>C7-D7</f>
-        <v>0</v>
+      <c r="E7" s="67" t="str">
+        <f>IF(A7="","",C7-D7)</f>
       </c>
       <c r="F7" s="68"/>
       <c r="G7" s="48" t="str">
-        <f>IF(ABS(E7)&lt;=F7,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A7="","",IF(OR(D7="",F7=""),"NOT READY",IF(ABS(E7)&lt;=F7,"PASS","REVIEW")))</f>
       </c>
       <c r="H7" s="50"/>
     </row>
     <row r="8">
       <c r="A8" s="50"/>
       <c r="B8" s="50"/>
-      <c r="C8" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A8)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A8)</f>
-        <v>0</v>
+      <c r="C8" s="67" t="str">
+        <f>IF(A8="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A8)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A8))</f>
       </c>
       <c r="D8" s="68"/>
-      <c r="E8" s="67" t="n">
-        <f>C8-D8</f>
-        <v>0</v>
+      <c r="E8" s="67" t="str">
+        <f>IF(A8="","",C8-D8)</f>
       </c>
       <c r="F8" s="68"/>
       <c r="G8" s="48" t="str">
-        <f>IF(ABS(E8)&lt;=F8,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A8="","",IF(OR(D8="",F8=""),"NOT READY",IF(ABS(E8)&lt;=F8,"PASS","REVIEW")))</f>
       </c>
       <c r="H8" s="50"/>
     </row>
     <row r="9">
       <c r="A9" s="50"/>
       <c r="B9" s="50"/>
-      <c r="C9" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A9)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A9)</f>
-        <v>0</v>
+      <c r="C9" s="67" t="str">
+        <f>IF(A9="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A9)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A9))</f>
       </c>
       <c r="D9" s="68"/>
-      <c r="E9" s="67" t="n">
-        <f>C9-D9</f>
-        <v>0</v>
+      <c r="E9" s="67" t="str">
+        <f>IF(A9="","",C9-D9)</f>
       </c>
       <c r="F9" s="68"/>
       <c r="G9" s="48" t="str">
-        <f>IF(ABS(E9)&lt;=F9,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A9="","",IF(OR(D9="",F9=""),"NOT READY",IF(ABS(E9)&lt;=F9,"PASS","REVIEW")))</f>
       </c>
       <c r="H9" s="50"/>
     </row>
     <row r="10">
       <c r="A10" s="50"/>
       <c r="B10" s="50"/>
-      <c r="C10" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A10)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A10)</f>
-        <v>0</v>
+      <c r="C10" s="67" t="str">
+        <f>IF(A10="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A10)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A10))</f>
       </c>
       <c r="D10" s="68"/>
-      <c r="E10" s="67" t="n">
-        <f>C10-D10</f>
-        <v>0</v>
+      <c r="E10" s="67" t="str">
+        <f>IF(A10="","",C10-D10)</f>
       </c>
       <c r="F10" s="68"/>
       <c r="G10" s="48" t="str">
-        <f>IF(ABS(E10)&lt;=F10,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A10="","",IF(OR(D10="",F10=""),"NOT READY",IF(ABS(E10)&lt;=F10,"PASS","REVIEW")))</f>
       </c>
       <c r="H10" s="50"/>
     </row>
     <row r="11">
       <c r="A11" s="50"/>
       <c r="B11" s="50"/>
-      <c r="C11" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A11)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A11)</f>
-        <v>0</v>
+      <c r="C11" s="67" t="str">
+        <f>IF(A11="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A11)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A11))</f>
       </c>
       <c r="D11" s="68"/>
-      <c r="E11" s="67" t="n">
-        <f>C11-D11</f>
-        <v>0</v>
+      <c r="E11" s="67" t="str">
+        <f>IF(A11="","",C11-D11)</f>
       </c>
       <c r="F11" s="68"/>
       <c r="G11" s="48" t="str">
-        <f>IF(ABS(E11)&lt;=F11,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A11="","",IF(OR(D11="",F11=""),"NOT READY",IF(ABS(E11)&lt;=F11,"PASS","REVIEW")))</f>
       </c>
       <c r="H11" s="50"/>
     </row>
     <row r="12">
       <c r="A12" s="50"/>
       <c r="B12" s="50"/>
-      <c r="C12" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A12)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A12)</f>
-        <v>0</v>
+      <c r="C12" s="67" t="str">
+        <f>IF(A12="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A12)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A12))</f>
       </c>
       <c r="D12" s="68"/>
-      <c r="E12" s="67" t="n">
-        <f>C12-D12</f>
-        <v>0</v>
+      <c r="E12" s="67" t="str">
+        <f>IF(A12="","",C12-D12)</f>
       </c>
       <c r="F12" s="68"/>
       <c r="G12" s="48" t="str">
-        <f>IF(ABS(E12)&lt;=F12,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A12="","",IF(OR(D12="",F12=""),"NOT READY",IF(ABS(E12)&lt;=F12,"PASS","REVIEW")))</f>
       </c>
       <c r="H12" s="50"/>
     </row>
     <row r="13">
       <c r="A13" s="50"/>
       <c r="B13" s="50"/>
-      <c r="C13" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A13)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A13)</f>
-        <v>0</v>
+      <c r="C13" s="67" t="str">
+        <f>IF(A13="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A13)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A13))</f>
       </c>
       <c r="D13" s="68"/>
-      <c r="E13" s="67" t="n">
-        <f>C13-D13</f>
-        <v>0</v>
+      <c r="E13" s="67" t="str">
+        <f>IF(A13="","",C13-D13)</f>
       </c>
       <c r="F13" s="68"/>
       <c r="G13" s="48" t="str">
-        <f>IF(ABS(E13)&lt;=F13,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A13="","",IF(OR(D13="",F13=""),"NOT READY",IF(ABS(E13)&lt;=F13,"PASS","REVIEW")))</f>
       </c>
       <c r="H13" s="50"/>
     </row>
     <row r="14">
       <c r="A14" s="50"/>
       <c r="B14" s="50"/>
-      <c r="C14" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A14)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A14)</f>
-        <v>0</v>
+      <c r="C14" s="67" t="str">
+        <f>IF(A14="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A14)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A14))</f>
       </c>
       <c r="D14" s="68"/>
-      <c r="E14" s="67" t="n">
-        <f>C14-D14</f>
-        <v>0</v>
+      <c r="E14" s="67" t="str">
+        <f>IF(A14="","",C14-D14)</f>
       </c>
       <c r="F14" s="68"/>
       <c r="G14" s="48" t="str">
-        <f>IF(ABS(E14)&lt;=F14,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A14="","",IF(OR(D14="",F14=""),"NOT READY",IF(ABS(E14)&lt;=F14,"PASS","REVIEW")))</f>
       </c>
       <c r="H14" s="50"/>
     </row>
     <row r="15">
       <c r="A15" s="50"/>
       <c r="B15" s="50"/>
-      <c r="C15" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A15)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A15)</f>
-        <v>0</v>
+      <c r="C15" s="67" t="str">
+        <f>IF(A15="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A15)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A15))</f>
       </c>
       <c r="D15" s="68"/>
-      <c r="E15" s="67" t="n">
-        <f>C15-D15</f>
-        <v>0</v>
+      <c r="E15" s="67" t="str">
+        <f>IF(A15="","",C15-D15)</f>
       </c>
       <c r="F15" s="68"/>
       <c r="G15" s="48" t="str">
-        <f>IF(ABS(E15)&lt;=F15,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A15="","",IF(OR(D15="",F15=""),"NOT READY",IF(ABS(E15)&lt;=F15,"PASS","REVIEW")))</f>
       </c>
       <c r="H15" s="50"/>
     </row>
     <row r="16">
       <c r="A16" s="50"/>
       <c r="B16" s="50"/>
-      <c r="C16" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A16)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A16)</f>
-        <v>0</v>
+      <c r="C16" s="67" t="str">
+        <f>IF(A16="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A16)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A16))</f>
       </c>
       <c r="D16" s="68"/>
-      <c r="E16" s="67" t="n">
-        <f>C16-D16</f>
-        <v>0</v>
+      <c r="E16" s="67" t="str">
+        <f>IF(A16="","",C16-D16)</f>
       </c>
       <c r="F16" s="68"/>
       <c r="G16" s="48" t="str">
-        <f>IF(ABS(E16)&lt;=F16,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A16="","",IF(OR(D16="",F16=""),"NOT READY",IF(ABS(E16)&lt;=F16,"PASS","REVIEW")))</f>
       </c>
       <c r="H16" s="50"/>
     </row>
     <row r="17">
       <c r="A17" s="50"/>
       <c r="B17" s="50"/>
-      <c r="C17" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A17)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A17)</f>
-        <v>0</v>
+      <c r="C17" s="67" t="str">
+        <f>IF(A17="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A17)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A17))</f>
       </c>
       <c r="D17" s="68"/>
-      <c r="E17" s="67" t="n">
-        <f>C17-D17</f>
-        <v>0</v>
+      <c r="E17" s="67" t="str">
+        <f>IF(A17="","",C17-D17)</f>
       </c>
       <c r="F17" s="68"/>
       <c r="G17" s="48" t="str">
-        <f>IF(ABS(E17)&lt;=F17,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A17="","",IF(OR(D17="",F17=""),"NOT READY",IF(ABS(E17)&lt;=F17,"PASS","REVIEW")))</f>
       </c>
       <c r="H17" s="50"/>
     </row>
     <row r="18">
       <c r="A18" s="50"/>
       <c r="B18" s="50"/>
-      <c r="C18" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A18)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A18)</f>
-        <v>0</v>
+      <c r="C18" s="67" t="str">
+        <f>IF(A18="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A18)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A18))</f>
       </c>
       <c r="D18" s="68"/>
-      <c r="E18" s="67" t="n">
-        <f>C18-D18</f>
-        <v>0</v>
+      <c r="E18" s="67" t="str">
+        <f>IF(A18="","",C18-D18)</f>
       </c>
       <c r="F18" s="68"/>
       <c r="G18" s="48" t="str">
-        <f>IF(ABS(E18)&lt;=F18,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A18="","",IF(OR(D18="",F18=""),"NOT READY",IF(ABS(E18)&lt;=F18,"PASS","REVIEW")))</f>
       </c>
       <c r="H18" s="50"/>
     </row>
     <row r="19">
       <c r="A19" s="50"/>
       <c r="B19" s="50"/>
-      <c r="C19" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A19)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A19)</f>
-        <v>0</v>
+      <c r="C19" s="67" t="str">
+        <f>IF(A19="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A19)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A19))</f>
       </c>
       <c r="D19" s="68"/>
-      <c r="E19" s="67" t="n">
-        <f>C19-D19</f>
-        <v>0</v>
+      <c r="E19" s="67" t="str">
+        <f>IF(A19="","",C19-D19)</f>
       </c>
       <c r="F19" s="68"/>
       <c r="G19" s="48" t="str">
-        <f>IF(ABS(E19)&lt;=F19,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A19="","",IF(OR(D19="",F19=""),"NOT READY",IF(ABS(E19)&lt;=F19,"PASS","REVIEW")))</f>
       </c>
       <c r="H19" s="50"/>
     </row>
     <row r="20">
       <c r="A20" s="50"/>
       <c r="B20" s="50"/>
-      <c r="C20" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A20)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A20)</f>
-        <v>0</v>
+      <c r="C20" s="67" t="str">
+        <f>IF(A20="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A20)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A20))</f>
       </c>
       <c r="D20" s="68"/>
-      <c r="E20" s="67" t="n">
-        <f>C20-D20</f>
-        <v>0</v>
+      <c r="E20" s="67" t="str">
+        <f>IF(A20="","",C20-D20)</f>
       </c>
       <c r="F20" s="68"/>
       <c r="G20" s="48" t="str">
-        <f>IF(ABS(E20)&lt;=F20,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A20="","",IF(OR(D20="",F20=""),"NOT READY",IF(ABS(E20)&lt;=F20,"PASS","REVIEW")))</f>
       </c>
       <c r="H20" s="50"/>
     </row>
     <row r="21">
       <c r="A21" s="50"/>
       <c r="B21" s="50"/>
-      <c r="C21" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A21)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A21)</f>
-        <v>0</v>
+      <c r="C21" s="67" t="str">
+        <f>IF(A21="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A21)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A21))</f>
       </c>
       <c r="D21" s="68"/>
-      <c r="E21" s="67" t="n">
-        <f>C21-D21</f>
-        <v>0</v>
+      <c r="E21" s="67" t="str">
+        <f>IF(A21="","",C21-D21)</f>
       </c>
       <c r="F21" s="68"/>
       <c r="G21" s="48" t="str">
-        <f>IF(ABS(E21)&lt;=F21,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A21="","",IF(OR(D21="",F21=""),"NOT READY",IF(ABS(E21)&lt;=F21,"PASS","REVIEW")))</f>
       </c>
       <c r="H21" s="50"/>
     </row>
     <row r="22">
       <c r="A22" s="50"/>
       <c r="B22" s="50"/>
-      <c r="C22" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A22)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A22)</f>
-        <v>0</v>
+      <c r="C22" s="67" t="str">
+        <f>IF(A22="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A22)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A22))</f>
       </c>
       <c r="D22" s="68"/>
-      <c r="E22" s="67" t="n">
-        <f>C22-D22</f>
-        <v>0</v>
+      <c r="E22" s="67" t="str">
+        <f>IF(A22="","",C22-D22)</f>
       </c>
       <c r="F22" s="68"/>
       <c r="G22" s="48" t="str">
-        <f>IF(ABS(E22)&lt;=F22,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A22="","",IF(OR(D22="",F22=""),"NOT READY",IF(ABS(E22)&lt;=F22,"PASS","REVIEW")))</f>
       </c>
       <c r="H22" s="50"/>
     </row>
     <row r="23">
       <c r="A23" s="50"/>
       <c r="B23" s="50"/>
-      <c r="C23" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A23)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A23)</f>
-        <v>0</v>
+      <c r="C23" s="67" t="str">
+        <f>IF(A23="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A23)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A23))</f>
       </c>
       <c r="D23" s="68"/>
-      <c r="E23" s="67" t="n">
-        <f>C23-D23</f>
-        <v>0</v>
+      <c r="E23" s="67" t="str">
+        <f>IF(A23="","",C23-D23)</f>
       </c>
       <c r="F23" s="68"/>
       <c r="G23" s="48" t="str">
-        <f>IF(ABS(E23)&lt;=F23,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A23="","",IF(OR(D23="",F23=""),"NOT READY",IF(ABS(E23)&lt;=F23,"PASS","REVIEW")))</f>
       </c>
       <c r="H23" s="50"/>
     </row>
     <row r="24">
       <c r="A24" s="50"/>
       <c r="B24" s="50"/>
-      <c r="C24" s="67" t="n">
-        <f>SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A24)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A24)</f>
-        <v>0</v>
+      <c r="C24" s="67" t="str">
+        <f>IF(A24="","",SUMIFS('Source_Data'!$F$5:$F$29,'Source_Data'!$C$5:$C$29,A24)-SUMIFS('Source_Data'!$G$5:$G$29,'Source_Data'!$C$5:$C$29,A24))</f>
       </c>
       <c r="D24" s="68"/>
-      <c r="E24" s="67" t="n">
-        <f>C24-D24</f>
-        <v>0</v>
+      <c r="E24" s="67" t="str">
+        <f>IF(A24="","",C24-D24)</f>
       </c>
       <c r="F24" s="68"/>
       <c r="G24" s="48" t="str">
-        <f>IF(ABS(E24)&lt;=F24,"PASS","REVIEW")</f>
-        <v>PASS</v>
+        <f>IF(A24="","",IF(OR(D24="",F24=""),"NOT READY",IF(ABS(E24)&lt;=F24,"PASS","REVIEW")))</f>
       </c>
       <c r="H24" s="50"/>
     </row>
@@ -2094,7 +2045,7 @@
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
-    <tablePart r:id="Rcceffbf57d5a4858"/>
+    <tablePart r:id="Re79f869f66194a62"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2340,7 +2291,7 @@
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
-    <tablePart r:id="Rade219d9bca34a54"/>
+    <tablePart r:id="R0dc8b4728cd442b2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2682,7 +2633,7 @@
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="portrait" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
-    <tablePart r:id="R3b6360dfbb604cd3"/>
+    <tablePart r:id="R939c1ad0b16f41cc"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2931,7 +2882,7 @@
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup paperSize="1" orientation="landscape" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
-    <tablePart r:id="Re299acbb085045ce"/>
+    <tablePart r:id="R62cec95be2364aea"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3003,14 +2954,14 @@
     </row>
     <row r="5">
       <c r="A5" s="48" t="str">
-        <v>Source debits equal source credits</v>
+        <v>Source population loaded</v>
       </c>
       <c r="B5" s="48" t="str">
-        <f>IF(C5=0,"PASS","FAIL")</f>
-        <v>PASS</v>
+        <f>IF(C5=0,"NOT READY","PASS")</f>
+        <v>NOT READY</v>
       </c>
       <c r="C5" s="48" t="n">
-        <f>SUM('Source_Data'!$F$5:$F$29)-SUM('Source_Data'!$G$5:$G$29)</f>
+        <f>COUNTA('Source_Data'!$A$5:$A$29)</f>
         <v>0</v>
       </c>
       <c r="D5" s="48" t="str">
@@ -3023,18 +2974,18 @@
     </row>
     <row r="6">
       <c r="A6" s="48" t="str">
-        <v>Proposed debits equal proposed credits</v>
+        <v>Source debits equal source credits</v>
       </c>
       <c r="B6" s="48" t="str">
-        <f>IF(C6=0,"PASS","FAIL")</f>
-        <v>PASS</v>
+        <f>IF(C5=0,"NOT READY",IF(ABS(C6)&lt;0.005,"PASS","FAIL"))</f>
+        <v>NOT READY</v>
       </c>
       <c r="C6" s="48" t="n">
-        <f>SUM('Proposed_Entries'!$D$5:$D$19)-SUM('Proposed_Entries'!$E$5:$E$19)</f>
+        <f>SUM('Source_Data'!$F$5:$F$29)-SUM('Source_Data'!$G$5:$G$29)</f>
         <v>0</v>
       </c>
       <c r="D6" s="48" t="str">
-        <v>Proposed_Entries</v>
+        <v>Source_Data</v>
       </c>
       <c r="E6" s="48"/>
       <c r="F6" s="48"/>
@@ -3043,18 +2994,18 @@
     </row>
     <row r="7">
       <c r="A7" s="48" t="str">
-        <v>No reconciliation rows require review</v>
+        <v>Account mapping loaded</v>
       </c>
       <c r="B7" s="48" t="str">
-        <f>IF(C7=0,"PASS","FAIL")</f>
-        <v>PASS</v>
+        <f>IF(C7=0,"NOT READY","PASS")</f>
+        <v>NOT READY</v>
       </c>
       <c r="C7" s="48" t="n">
-        <f>COUNTIF('Reconciliation'!$G$5:$G$24,"REVIEW")</f>
+        <f>COUNTA('Account_Map'!$A$5:$A$29)</f>
         <v>0</v>
       </c>
       <c r="D7" s="48" t="str">
-        <v>Reconciliation</v>
+        <v>Account_Map</v>
       </c>
       <c r="E7" s="48"/>
       <c r="F7" s="48"/>
@@ -3063,18 +3014,18 @@
     </row>
     <row r="8">
       <c r="A8" s="48" t="str">
-        <v>No open exceptions</v>
+        <v>Reconciliation rows complete and passing</v>
       </c>
       <c r="B8" s="48" t="str">
-        <f>IF(C8=0,"PASS","FAIL")</f>
-        <v>PASS</v>
+        <f>IF(COUNTA('Reconciliation'!$A$5:$A$24)=0,"NOT READY",IF(C8=0,"PASS","FAIL"))</f>
+        <v>NOT READY</v>
       </c>
       <c r="C8" s="48" t="n">
-        <f>COUNTIF('Exceptions'!$G$5:$G$19,"Open")</f>
+        <f>COUNTA('Reconciliation'!$A$5:$A$24)-COUNTIF('Reconciliation'!$G$5:$G$24,"PASS")</f>
         <v>0</v>
       </c>
       <c r="D8" s="48" t="str">
-        <v>Exceptions</v>
+        <v>Reconciliation</v>
       </c>
       <c r="E8" s="48"/>
       <c r="F8" s="48"/>
@@ -3083,18 +3034,18 @@
     </row>
     <row r="9">
       <c r="A9" s="48" t="str">
-        <v>Required close fields populated</v>
+        <v>Proposed entries balanced when present</v>
       </c>
       <c r="B9" s="48" t="str">
-        <f>IF(C9=0,"PASS","FAIL")</f>
-        <v>FAIL</v>
+        <f>IF(COUNTA('Proposed_Entries'!$A$5:$A$19)=0,"NOT APPLICABLE",IF(ABS(C9)&lt;0.005,"PASS","FAIL"))</f>
+        <v>NOT APPLICABLE</v>
       </c>
       <c r="C9" s="48" t="n">
-        <f>IF(OR('Close_Control'!B5="{{organization_name}}",'Close_Control'!B6="{{close_period_end}}",'Close_Control'!B7="{{preparer_role}}",'Close_Control'!B8="{{reviewer_role}}"),1,0)</f>
-        <v>1</v>
+        <f>SUM('Proposed_Entries'!$D$5:$D$19)-SUM('Proposed_Entries'!$E$5:$E$19)</f>
+        <v>0</v>
       </c>
       <c r="D9" s="48" t="str">
-        <v>Close_Control</v>
+        <v>Proposed_Entries</v>
       </c>
       <c r="E9" s="48"/>
       <c r="F9" s="48"/>
@@ -3102,37 +3053,48 @@
       <c r="H9" s="48"/>
     </row>
     <row r="10">
-      <c r="A10" s="48"/>
-      <c r="B10" s="48"/>
-      <c r="C10" s="48"/>
-      <c r="D10" s="48"/>
+      <c r="A10" s="48" t="str">
+        <v>No open exceptions</v>
+      </c>
+      <c r="B10" s="48" t="str">
+        <f>IF(COUNTA('Reconciliation'!$A$5:$A$24)=0,"NOT READY",IF(C10=0,"PASS","FAIL"))</f>
+        <v>NOT READY</v>
+      </c>
+      <c r="C10" s="48" t="n">
+        <f>COUNTIF('Exceptions'!$G$5:$G$19,"Open")</f>
+        <v>0</v>
+      </c>
+      <c r="D10" s="48" t="str">
+        <v>Exceptions</v>
+      </c>
       <c r="E10" s="48"/>
       <c r="F10" s="48"/>
       <c r="G10" s="48"/>
       <c r="H10" s="48"/>
     </row>
     <row r="11">
-      <c r="A11" s="49" t="str">
-        <v>MODEL STATUS</v>
-      </c>
-      <c r="B11" s="49" t="str">
-        <v>Formula</v>
-      </c>
-      <c r="C11" s="48"/>
-      <c r="D11" s="48"/>
+      <c r="A11" s="48" t="str">
+        <v>Required close fields populated</v>
+      </c>
+      <c r="B11" s="48" t="str">
+        <f>IF(C11=0,"PASS","NOT READY")</f>
+        <v>NOT READY</v>
+      </c>
+      <c r="C11" s="48" t="n">
+        <f>IF(OR(COUNTBLANK('Close_Control'!B5:B8)&gt;0,LEFT('Close_Control'!B5,1)="{",LEFT('Close_Control'!B6,1)="{",LEFT('Close_Control'!B7,1)="{",LEFT('Close_Control'!B8,1)="{"),1,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D11" s="48" t="str">
+        <v>Close_Control</v>
+      </c>
       <c r="E11" s="48"/>
       <c r="F11" s="48"/>
       <c r="G11" s="48"/>
       <c r="H11" s="48"/>
     </row>
     <row r="12">
-      <c r="A12" s="48" t="str">
-        <v>Status</v>
-      </c>
-      <c r="B12" s="70" t="str">
-        <f>IF(COUNTIF(B5:B9,"FAIL")=0,"PASS","FAIL")</f>
-        <v>FAIL</v>
-      </c>
+      <c r="A12" s="48"/>
+      <c r="B12" s="48"/>
       <c r="C12" s="48"/>
       <c r="D12" s="48"/>
       <c r="E12" s="48"/>
@@ -3140,14 +3102,44 @@
       <c r="G12" s="48"/>
       <c r="H12" s="48"/>
     </row>
+    <row r="13">
+      <c r="A13" s="49" t="str">
+        <v>MODEL STATUS</v>
+      </c>
+      <c r="B13" s="49" t="str">
+        <v>Formula</v>
+      </c>
+      <c r="C13" s="48"/>
+      <c r="D13" s="48"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="48"/>
+      <c r="G13" s="48"/>
+      <c r="H13" s="48"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="48" t="str">
+        <v>Status</v>
+      </c>
+      <c r="B14" s="70" t="str">
+        <f>IF(AND(COUNTIF(B5:B11,"NOT READY")=0,COUNTIF(B5:B11,"FAIL")=0),"PASS","NOT READY")</f>
+        <v>NOT READY</v>
+      </c>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="48"/>
+    </row>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B9">
+  <conditionalFormatting sqref="B5:B11">
     <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="PASS"/>
     <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="FAIL"/>
+    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="NOT READY"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>

</xml_diff>

<commit_message>
fix: close workbook integrity and scale gates
</commit_message>
<xml_diff>
--- a/library/templates/TMPL-0001/1.0.0/internal-close-reconciliation.xlsx
+++ b/library/templates/TMPL-0001/1.0.0/internal-close-reconciliation.xlsx
@@ -27,7 +27,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Exceptions'!$A$1:$H$19</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Checks'!$A$1:$D$16</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
   <extLst>
     <ext uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <ns2:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
@@ -270,7 +270,7 @@
     <t xml:space="preserve">Source debits equal source credits</t>
   </si>
   <si>
-    <t xml:space="preserve">Account mapping rows complete</t>
+    <t xml:space="preserve">Account mappings complete; source covered</t>
   </si>
   <si>
     <t xml:space="preserve">Account_Map</t>
@@ -279,13 +279,13 @@
     <t xml:space="preserve">Reconciliation inputs complete and passing</t>
   </si>
   <si>
-    <t xml:space="preserve">Proposed entries balanced when present</t>
+    <t xml:space="preserve">Proposed entries complete and balanced</t>
   </si>
   <si>
     <t xml:space="preserve">Proposed_Entries</t>
   </si>
   <si>
-    <t xml:space="preserve">No open exceptions</t>
+    <t xml:space="preserve">Exceptions valid; none open</t>
   </si>
   <si>
     <t xml:space="preserve">Exceptions</t>
@@ -3477,7 +3477,7 @@
         <v>NOT READY</v>
       </c>
       <c r="C8" s="3" t="n">
-        <f aca="false">SUMPRODUCT(--(((Account_Map!$A$5:$A$29&lt;&gt;"")+(Account_Map!$B$5:$B$29&lt;&gt;"")+(Account_Map!$C$5:$C$29&lt;&gt;"")+(Account_Map!$D$5:$D$29&lt;&gt;"")+(Account_Map!$E$5:$E$29&lt;&gt;""))&gt;0))-SUMPRODUCT(--(Account_Map!$A$5:$A$29&lt;&gt;""),--(Account_Map!$B$5:$B$29&lt;&gt;""),--(Account_Map!$C$5:$C$29&lt;&gt;""),--(Account_Map!$D$5:$D$29&lt;&gt;""),--(((Account_Map!$E$5:$E$29="Yes")+(Account_Map!$E$5:$E$29="No"))&gt;0))</f>
+        <f aca="false">SUMPRODUCT(--(((Account_Map!$A$5:$A$29&lt;&gt;"")+(Account_Map!$B$5:$B$29&lt;&gt;"")+(Account_Map!$C$5:$C$29&lt;&gt;"")+(Account_Map!$D$5:$D$29&lt;&gt;"")+(Account_Map!$E$5:$E$29&lt;&gt;""))&gt;0))-SUMPRODUCT(--(Account_Map!$A$5:$A$29&lt;&gt;""),--(Account_Map!$B$5:$B$29&lt;&gt;""),--(Account_Map!$C$5:$C$29&lt;&gt;""),--(Account_Map!$D$5:$D$29&lt;&gt;""),--(((Account_Map!$E$5:$E$29="Yes")+(Account_Map!$E$5:$E$29="No"))&gt;0))+SUMPRODUCT(--(Source_Data!$C$5:$C$29&lt;&gt;""),--(COUNTIFS(Account_Map!$A$5:$A$29,Source_Data!$C$5:$C$29,Account_Map!$E$5:$E$29,"Yes")&lt;&gt;1))</f>
         <v>0</v>
       </c>
       <c r="D8" s="3" t="s">
@@ -3513,11 +3513,11 @@
         <v>80</v>
       </c>
       <c r="B10" s="3" t="str">
-        <f aca="false">IF(COUNTA(Proposed_Entries!$A$5:$A$19)=0,"NOT APPLICABLE",IF(ABS(C10)&lt;0.005,"PASS","FAIL"))</f>
+        <f aca="false">IF(SUMPRODUCT(--(((Proposed_Entries!$A$5:$A$19&lt;&gt;"")+(Proposed_Entries!$B$5:$B$19&lt;&gt;"")+(Proposed_Entries!$C$5:$C$19&lt;&gt;"")+(Proposed_Entries!$D$5:$D$19&lt;&gt;"")+(Proposed_Entries!$E$5:$E$19&lt;&gt;"")+(Proposed_Entries!$F$5:$F$19&lt;&gt;"")+(Proposed_Entries!$G$5:$G$19&lt;&gt;"")+(Proposed_Entries!$H$5:$H$19&lt;&gt;""))&gt;0))=0,"NOT APPLICABLE",IF(C10=0,"PASS","FAIL"))</f>
         <v>NOT APPLICABLE</v>
       </c>
       <c r="C10" s="3" t="n">
-        <f aca="false">SUM(Proposed_Entries!$D$5:$D$19)-SUM(Proposed_Entries!$E$5:$E$19)</f>
+        <f aca="false">SUMPRODUCT(--(((Proposed_Entries!$A$5:$A$19&lt;&gt;"")+(Proposed_Entries!$B$5:$B$19&lt;&gt;"")+(Proposed_Entries!$C$5:$C$19&lt;&gt;"")+(Proposed_Entries!$D$5:$D$19&lt;&gt;"")+(Proposed_Entries!$E$5:$E$19&lt;&gt;"")+(Proposed_Entries!$F$5:$F$19&lt;&gt;"")+(Proposed_Entries!$G$5:$G$19&lt;&gt;"")+(Proposed_Entries!$H$5:$H$19&lt;&gt;""))&gt;0))-SUMPRODUCT(--(Proposed_Entries!$A$5:$A$19&lt;&gt;""),--(Proposed_Entries!$B$5:$B$19&lt;&gt;""),--(Proposed_Entries!$C$5:$C$19&lt;&gt;""),--ISNUMBER(Proposed_Entries!$D$5:$D$19),--ISNUMBER(Proposed_Entries!$E$5:$E$19),--(Proposed_Entries!$F$5:$F$19&lt;&gt;""),--(((Proposed_Entries!$G$5:$G$19="Draft")+(Proposed_Entries!$G$5:$G$19="Ready for review")+(Proposed_Entries!$G$5:$G$19="Hold"))&gt;0))+IF(ABS(SUM(Proposed_Entries!$D$5:$D$19)-SUM(Proposed_Entries!$E$5:$E$19))&lt;0.005,0,1)</f>
         <v>0</v>
       </c>
       <c r="D10" s="3" t="s">
@@ -3537,7 +3537,7 @@
         <v>NOT READY</v>
       </c>
       <c r="C11" s="3" t="n">
-        <f aca="false">COUNTIF(Exceptions!$G$5:$G$19,"Open")</f>
+        <f aca="false">SUMPRODUCT(--(((Exceptions!$A$5:$A$19&lt;&gt;"")+(Exceptions!$B$5:$B$19&lt;&gt;"")+(Exceptions!$C$5:$C$19&lt;&gt;"")+(Exceptions!$D$5:$D$19&lt;&gt;"")+(Exceptions!$E$5:$E$19&lt;&gt;"")+(Exceptions!$F$5:$F$19&lt;&gt;"")+(Exceptions!$G$5:$G$19&lt;&gt;"")+(Exceptions!$H$5:$H$19&lt;&gt;""))&gt;0))-SUMPRODUCT(--(Exceptions!$A$5:$A$19&lt;&gt;""),--(Exceptions!$B$5:$B$19&lt;&gt;""),--(Exceptions!$C$5:$C$19&lt;&gt;""),--(((Exceptions!$D$5:$D$19="supporting")+(Exceptions!$D$5:$D$19="contextual")+(Exceptions!$D$5:$D$19="question-only")+(Exceptions!$D$5:$D$19="superseded"))&gt;0),--(Exceptions!$E$5:$E$19&lt;&gt;""),--ISNUMBER(Exceptions!$F$5:$F$19),--(((Exceptions!$G$5:$G$19="Open")+(Exceptions!$G$5:$G$19="Resolved")+(Exceptions!$G$5:$G$19="Retained"))&gt;0),--(((Exceptions!$G$5:$G$19&lt;&gt;"Resolved")+(Exceptions!$H$5:$H$19&lt;&gt;""))&gt;0))+COUNTIF(Exceptions!$G$5:$G$19,"Open")</f>
         <v>0</v>
       </c>
       <c r="D11" s="3" t="s">

</xml_diff>

<commit_message>
fix: bind reconciliation to source coverage
</commit_message>
<xml_diff>
--- a/library/templates/TMPL-0001/1.0.0/internal-close-reconciliation.xlsx
+++ b/library/templates/TMPL-0001/1.0.0/internal-close-reconciliation.xlsx
@@ -276,7 +276,7 @@
     <t xml:space="preserve">Account_Map</t>
   </si>
   <si>
-    <t xml:space="preserve">Reconciliation inputs complete and passing</t>
+    <t xml:space="preserve">Reconciliation complete; mapped and source-covered</t>
   </si>
   <si>
     <t xml:space="preserve">Proposed entries complete and balanced</t>
@@ -3497,7 +3497,7 @@
         <v>NOT READY</v>
       </c>
       <c r="C9" s="3" t="n">
-        <f aca="false">SUMPRODUCT(--(((Reconciliation!$A$5:$A$24&lt;&gt;"")+(Reconciliation!$B$5:$B$24&lt;&gt;"")+(Reconciliation!$D$5:$D$24&lt;&gt;"")+(Reconciliation!$F$5:$F$24&lt;&gt;"")+(Reconciliation!$H$5:$H$24&lt;&gt;""))&gt;0))-SUMPRODUCT(--(Reconciliation!$A$5:$A$24&lt;&gt;""),--(Reconciliation!$B$5:$B$24&lt;&gt;""),--ISNUMBER(Reconciliation!$D$5:$D$24),--ISNUMBER(Reconciliation!$F$5:$F$24),--(Reconciliation!$G$5:$G$24="PASS"))</f>
+        <f aca="false">SUMPRODUCT(--(((Reconciliation!$A$5:$A$24&lt;&gt;"")+(Reconciliation!$B$5:$B$24&lt;&gt;"")+(Reconciliation!$D$5:$D$24&lt;&gt;"")+(Reconciliation!$F$5:$F$24&lt;&gt;"")+(Reconciliation!$H$5:$H$24&lt;&gt;""))&gt;0))-SUMPRODUCT(--(Reconciliation!$A$5:$A$24&lt;&gt;""),--(Reconciliation!$B$5:$B$24&lt;&gt;""),--ISNUMBER(Reconciliation!$D$5:$D$24),--ISNUMBER(Reconciliation!$F$5:$F$24),--(Reconciliation!$G$5:$G$24="PASS"))+SUMPRODUCT(--(Source_Data!$C$5:$C$29&lt;&gt;""),--(COUNTIF(Reconciliation!$A$5:$A$24,Source_Data!$C$5:$C$29)&lt;&gt;1))+SUMPRODUCT(--(Reconciliation!$A$5:$A$24&lt;&gt;""),--(COUNTIFS(Account_Map!$A$5:$A$29,Reconciliation!$A$5:$A$24,Account_Map!$E$5:$E$29,"Yes")&lt;&gt;1))+SUMPRODUCT(--(Reconciliation!$A$5:$A$24&lt;&gt;""),--(COUNTIF(Source_Data!$C$5:$C$29,Reconciliation!$A$5:$A$24)=0))</f>
         <v>0</v>
       </c>
       <c r="D9" s="3" t="s">

</xml_diff>